<commit_message>
modify the promte very specific to the pdf type and add readme.md
</commit_message>
<xml_diff>
--- a/output/na_results.xlsx
+++ b/output/na_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,30 +434,35 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
+          <t>Block Number</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>Area in NA Order</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Dated</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>NA Order No.</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Lease Deed Doc. No.</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t xml:space="preserve">Lease Area </t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t xml:space="preserve">Lease Start </t>
         </is>
@@ -468,37 +473,30 @@
       <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>34576</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>08/01/2026</t>
-        </is>
-      </c>
+          <t>251/p2</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>IORA/31/02/112/9/2026</t>
+          <t>16/02/2026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>838/2025</t>
+          <t>IORA/31/02/112/25/2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>34576</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>28/05/2025</t>
+          <t>1141/2026</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>21/01/2026</t>
         </is>
       </c>
     </row>
@@ -507,29 +505,38 @@
       <c r="B3" t="inlineStr"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>251/p2</t>
+          <t>255</t>
         </is>
       </c>
       <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>34576</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>IORA/31/02/112/25/2026</t>
+          <t>08/01/2026</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1141/2026</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr"/>
+          <t>IORA/31/02/112/9/2026</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>838/2025</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>21/01/2026</t>
+          <t>34576</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>28/05/2025</t>
         </is>
       </c>
     </row>
@@ -541,32 +548,33 @@
           <t>256</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr">
         <is>
           <t>16510</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>07/01/2026</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>IORA/31/02/112/8/2026</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>854/2025</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>16510</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>28/05/2025</t>
         </is>
@@ -580,32 +588,33 @@
           <t>257</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr">
         <is>
           <t>16534</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>07/01/2026</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>IORA/31/02/112/7/2026</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>837/2025</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>16534</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>28/05/2025</t>
         </is>

</xml_diff>

<commit_message>
final modify output file collumn
</commit_message>
<xml_diff>
--- a/output/na_results.xlsx
+++ b/output/na_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,187 +434,218 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Block Number</t>
+          <t>Area in NA Order</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Area in NA Order</t>
+          <t>Dated</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Dated</t>
+          <t>NA Order No.</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>NA Order No.</t>
+          <t>Lease Deed Doc. No.</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Lease Deed Doc. No.</t>
+          <t xml:space="preserve">Lease Area </t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Lease Area </t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
         <is>
           <t xml:space="preserve">Lease Start </t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Rampura Mota</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>251/p2</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>5997.00</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>16/02/2026</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>16/02/2026</t>
+          <t>IORA/31/02/112/25/2026</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>IORA/31/02/112/25/2026</t>
+          <t>1141/2026</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1141/2026</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr">
+          <t>5997.00</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>21/01/2026</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Rampura Mota</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>255</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>34576</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t>08/01/2026</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>IORA/31/02/112/9/2026</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>838/2025</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>34576</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>08/01/2026</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>IORA/31/02/112/9/2026</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>838/2025</t>
-        </is>
-      </c>
       <c r="I3" t="inlineStr">
-        <is>
-          <t>34576</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
         <is>
           <t>28/05/2025</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
-      <c r="B4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Rampura Mota</t>
+        </is>
+      </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>256</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>16510</t>
+        </is>
+      </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>IORA/31/02/112/8/2026</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>854/2025</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>16510</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>07/01/2026</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>IORA/31/02/112/8/2026</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>854/2025</t>
-        </is>
-      </c>
       <c r="I4" t="inlineStr">
-        <is>
-          <t>16510</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
         <is>
           <t>28/05/2025</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr"/>
-      <c r="B5" t="inlineStr"/>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Rampura Mota</t>
+        </is>
+      </c>
       <c r="C5" t="inlineStr">
         <is>
           <t>257</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>16534</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t>07/01/2026</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>IORA/31/02/112/7/2026</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>837/2025</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>16534</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>07/01/2026</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>IORA/31/02/112/7/2026</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>837/2025</t>
-        </is>
-      </c>
       <c r="I5" t="inlineStr">
-        <is>
-          <t>16534</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
         <is>
           <t>28/05/2025</t>
         </is>

</xml_diff>

<commit_message>
correct for correcting the missing field value
</commit_message>
<xml_diff>
--- a/output/na_results.xlsx
+++ b/output/na_results.xlsx
@@ -548,7 +548,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>34576</t>
+          <t>16888</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -595,7 +595,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>16510</t>
+          <t>16959</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>16534</t>
+          <t>16534.00</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">

</xml_diff>

<commit_message>
partially ok for lease area
</commit_message>
<xml_diff>
--- a/output/na_results.xlsx
+++ b/output/na_results.xlsx
@@ -481,7 +481,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>5997.00</t>
+          <t>5997</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -499,11 +499,7 @@
           <t>1141/2026</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>5997.00</t>
-        </is>
-      </c>
+      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>21/01/2026</t>
@@ -642,7 +638,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>16534.00</t>
+          <t>16792</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">

</xml_diff>